<commit_message>
Item.xlsx(Weapon·Armor·Consumable) 추가, 상시 데이터에서 Active 열 제거
- Weapon 탭에 ItemType 열, Armor·Consumable 탭 열 구조(초안) 추가 → tables/Item.xlsx 한 파일
- enum 값(ItemType·ArmorSlot·ConsumableType 등)을 시트 1행과 구글 시트 README에 명시
- Active 열은 REGISTRY·Stage에만 남기고 나머지 시트에서 삭제
- REGISTRY: Weapon File=Item, Armor(14001~)·Consumable(15001~) 행 추가
- 열 구조가 바뀐 예전 csv/ 추출본 삭제

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CDH3mwZmVtgx1ALhFj2DHN
</commit_message>
<xml_diff>
--- a/tables/Attack.xlsx
+++ b/tables/Attack.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16.38" customWidth="1" min="1" max="1"/>
@@ -652,11 +652,6 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="inlineStr">
-        <is>
           <t>Note</t>
         </is>
       </c>
@@ -708,11 +703,6 @@
       <c r="N7" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="O7" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -761,11 +751,6 @@
       <c r="N8" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="O8" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -816,11 +801,6 @@
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="P9" s="3" t="inlineStr">
-        <is>
           <t>콤보 끝</t>
         </is>
       </c>
@@ -872,11 +852,6 @@
       <c r="N10" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="O10" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -927,11 +902,6 @@
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="P11" s="3" t="inlineStr">
-        <is>
           <t>잡몹 즉사, 보스는 Boss.ExecuteDamage. 회피 불가</t>
         </is>
       </c>
@@ -985,11 +955,6 @@
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="P12" s="3" t="inlineStr">
-        <is>
           <t>회피 불가, 결박 끊기</t>
         </is>
       </c>
@@ -1038,11 +1003,6 @@
       <c r="N13" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="O13" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -1090,11 +1050,6 @@
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="P14" s="3" t="inlineStr">
-        <is>
           <t>구속 1000ms, 공격 연타로 풀기</t>
         </is>
       </c>
@@ -1143,11 +1098,6 @@
       <c r="N15" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="O15" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -1195,11 +1145,6 @@
       </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="P16" s="3" t="inlineStr">
-        <is>
           <t>슈퍼아머, 벽 충돌 시 800ms 허점</t>
         </is>
       </c>
@@ -1250,11 +1195,6 @@
       </c>
       <c r="O17" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="P17" s="3" t="inlineStr">
-        <is>
           <t>초당 고정 5 피해, 3000ms</t>
         </is>
       </c>
@@ -1305,11 +1245,6 @@
       </c>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="P18" s="3" t="inlineStr">
-        <is>
           <t>포물선</t>
         </is>
       </c>
@@ -1358,11 +1293,6 @@
       <c r="N19" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="O19" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -1410,11 +1340,6 @@
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="P20" s="3" t="inlineStr">
-        <is>
           <t>2타(어택 2-1)</t>
         </is>
       </c>
@@ -1465,11 +1390,6 @@
       </c>
       <c r="O21" s="3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="P21" s="3" t="inlineStr">
-        <is>
           <t>구속, 결박 가르기로 끊기</t>
         </is>
       </c>
@@ -1519,11 +1439,6 @@
         <v>100</v>
       </c>
       <c r="O22" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="P22" s="3" t="inlineStr">
         <is>
           <t>HP 50% 이하, 벽 충돌 시 보스 체세 -30</t>
         </is>

</xml_diff>